<commit_message>
feat: conexao TB vendedor por cliente
</commit_message>
<xml_diff>
--- a/Dados/acessos.xlsx
+++ b/Dados/acessos.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Drives compartilhados\BI - JLeandro Gestao\Moreira\01.Comercial\Dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77353992-1F86-477D-9BDA-04CE733ABC46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F7E98AA-6EA7-4C30-9619-F5E837788481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="10">
   <si>
     <t>acesso</t>
   </si>
@@ -37,6 +37,24 @@
   </si>
   <si>
     <t>Sabrina</t>
+  </si>
+  <si>
+    <t>vendedor</t>
+  </si>
+  <si>
+    <t>Paulo</t>
+  </si>
+  <si>
+    <t>INDUSTRIA</t>
+  </si>
+  <si>
+    <t>MARCELO</t>
+  </si>
+  <si>
+    <t>TINO</t>
+  </si>
+  <si>
+    <t>EWERTON</t>
   </si>
 </sst>
 </file>
@@ -354,31 +372,158 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>1230</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>1230</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>1230</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="B5">
         <v>3477</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <v>3477</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>3477</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8">
+        <v>3477</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9">
+        <v>3477</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
+      <c r="B10">
         <v>9480</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>9480</v>
+      </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12">
+        <v>9480</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13">
+        <v>9480</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <v>9480</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>